<commit_message>
update testcase + PCM
</commit_message>
<xml_diff>
--- a/SCI_SE_8.3.ProjectTestCaseSprint3.xlsx
+++ b/SCI_SE_8.3.ProjectTestCaseSprint3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\nhi\Khóa luận tốt nghiệp\Bao cao Su dung cho de tai nhom - Copy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\nhi\Khóa luận tốt nghiệp\Bao cao Su dung cho de tai nhom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ADFA939-F695-4306-A1DE-A3CBBCFC35FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A44C87-6CA6-44B4-AE56-F35A51F31998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" tabRatio="858" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" tabRatio="858" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trường hợp kiểm thử" sheetId="12" r:id="rId1"/>
@@ -1473,6 +1473,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1559,9 +1562,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1569,547 +1569,7 @@
     <cellStyle name="Normal 10" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal_Sheet1" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="102">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="48">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3185,47 +2645,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.05" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="52" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
     </row>
     <row r="2" spans="1:5" ht="11.3" customHeight="1">
-      <c r="A2" s="53"/>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
+      <c r="A2" s="54"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
     </row>
     <row r="3" spans="1:5" ht="42.75" customHeight="1">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="56" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="55"/>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
+      <c r="A4" s="56"/>
+      <c r="B4" s="56"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
     </row>
     <row r="5" spans="1:5" ht="38.200000000000003" customHeight="1">
       <c r="A5" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="56" t="s">
+      <c r="B5" s="57" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="59"/>
     </row>
     <row r="6" spans="1:5" ht="33.85">
       <c r="A6" s="7" t="s">
@@ -3255,9 +2715,9 @@
         <v>46</v>
       </c>
       <c r="D7" s="3">
-        <v>32</v>
-      </c>
-      <c r="E7" s="49" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="50" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3272,9 +2732,9 @@
         <v>45</v>
       </c>
       <c r="D8" s="3">
-        <v>26</v>
-      </c>
-      <c r="E8" s="50"/>
+        <v>39</v>
+      </c>
+      <c r="E8" s="51"/>
     </row>
     <row r="9" spans="1:5" ht="16.899999999999999">
       <c r="A9" s="3">
@@ -3287,9 +2747,9 @@
         <v>43</v>
       </c>
       <c r="D9" s="3">
-        <v>17</v>
-      </c>
-      <c r="E9" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="50" t="s">
         <v>23</v>
       </c>
     </row>
@@ -3304,14 +2764,14 @@
         <v>44</v>
       </c>
       <c r="D10" s="3">
-        <v>12</v>
-      </c>
-      <c r="E10" s="50"/>
+        <v>19</v>
+      </c>
+      <c r="E10" s="51"/>
     </row>
     <row r="11" spans="1:5" ht="16.899999999999999">
       <c r="D11" s="2">
         <f>+SUM(D7:D10)</f>
-        <v>87</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16.899999999999999">
@@ -3356,25 +2816,25 @@
       <c r="A1" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
     </row>
     <row r="2" spans="1:6" ht="16.899999999999999">
       <c r="A2" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="64" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
     </row>
     <row r="3" spans="1:6" ht="16.899999999999999">
       <c r="A3" s="39"/>
@@ -3435,64 +2895,64 @@
       </c>
     </row>
     <row r="30" spans="1:13" ht="16.899999999999999">
-      <c r="A30" s="61" t="s">
+      <c r="A30" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="B30" s="61" t="s">
+      <c r="B30" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="C30" s="61" t="s">
+      <c r="C30" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="D30" s="61" t="s">
+      <c r="D30" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="E30" s="61" t="s">
+      <c r="E30" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="F30" s="61" t="s">
+      <c r="F30" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="G30" s="61" t="s">
+      <c r="G30" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="H30" s="61"/>
-      <c r="I30" s="61"/>
-      <c r="J30" s="61" t="s">
+      <c r="H30" s="62"/>
+      <c r="I30" s="62"/>
+      <c r="J30" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="K30" s="61"/>
-      <c r="L30" s="61"/>
-      <c r="M30" s="61" t="s">
+      <c r="K30" s="62"/>
+      <c r="L30" s="62"/>
+      <c r="M30" s="62" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="16.899999999999999">
-      <c r="A31" s="61"/>
-      <c r="B31" s="61"/>
-      <c r="C31" s="61"/>
-      <c r="D31" s="61"/>
-      <c r="E31" s="61"/>
-      <c r="F31" s="61"/>
-      <c r="G31" s="61" t="s">
+      <c r="A31" s="62"/>
+      <c r="B31" s="62"/>
+      <c r="C31" s="62"/>
+      <c r="D31" s="62"/>
+      <c r="E31" s="62"/>
+      <c r="F31" s="62"/>
+      <c r="G31" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="H31" s="61"/>
-      <c r="I31" s="61"/>
-      <c r="J31" s="61" t="s">
+      <c r="H31" s="62"/>
+      <c r="I31" s="62"/>
+      <c r="J31" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="K31" s="61"/>
-      <c r="L31" s="61"/>
-      <c r="M31" s="61"/>
+      <c r="K31" s="62"/>
+      <c r="L31" s="62"/>
+      <c r="M31" s="62"/>
     </row>
     <row r="32" spans="1:13" ht="50.75">
-      <c r="A32" s="61"/>
-      <c r="B32" s="61"/>
-      <c r="C32" s="61"/>
-      <c r="D32" s="61"/>
-      <c r="E32" s="61"/>
-      <c r="F32" s="61"/>
+      <c r="A32" s="62"/>
+      <c r="B32" s="62"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="62"/>
       <c r="G32" s="24" t="s">
         <v>20</v>
       </c>
@@ -3511,24 +2971,24 @@
       <c r="L32" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="M32" s="61"/>
+      <c r="M32" s="62"/>
     </row>
     <row r="33" spans="1:13" ht="16.899999999999999">
-      <c r="A33" s="59" t="s">
+      <c r="A33" s="60" t="s">
         <v>50</v>
       </c>
-      <c r="B33" s="59"/>
-      <c r="C33" s="59"/>
-      <c r="D33" s="59"/>
-      <c r="E33" s="59"/>
-      <c r="F33" s="59"/>
-      <c r="G33" s="59"/>
-      <c r="H33" s="59"/>
-      <c r="I33" s="59"/>
-      <c r="J33" s="59"/>
-      <c r="K33" s="59"/>
-      <c r="L33" s="59"/>
-      <c r="M33" s="59"/>
+      <c r="B33" s="60"/>
+      <c r="C33" s="60"/>
+      <c r="D33" s="60"/>
+      <c r="E33" s="60"/>
+      <c r="F33" s="60"/>
+      <c r="G33" s="60"/>
+      <c r="H33" s="60"/>
+      <c r="I33" s="60"/>
+      <c r="J33" s="60"/>
+      <c r="K33" s="60"/>
+      <c r="L33" s="60"/>
+      <c r="M33" s="60"/>
     </row>
     <row r="34" spans="1:13" ht="33.85">
       <c r="A34" s="22" t="s">
@@ -4024,21 +3484,21 @@
       <c r="M50" s="12"/>
     </row>
     <row r="52" spans="1:13" ht="16.899999999999999">
-      <c r="A52" s="60" t="s">
+      <c r="A52" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="B52" s="60"/>
-      <c r="C52" s="60"/>
-      <c r="D52" s="60"/>
-      <c r="E52" s="60"/>
-      <c r="F52" s="60"/>
-      <c r="G52" s="60"/>
-      <c r="H52" s="60"/>
-      <c r="I52" s="60"/>
-      <c r="J52" s="60"/>
-      <c r="K52" s="60"/>
-      <c r="L52" s="60"/>
-      <c r="M52" s="60"/>
+      <c r="B52" s="61"/>
+      <c r="C52" s="61"/>
+      <c r="D52" s="61"/>
+      <c r="E52" s="61"/>
+      <c r="F52" s="61"/>
+      <c r="G52" s="61"/>
+      <c r="H52" s="61"/>
+      <c r="I52" s="61"/>
+      <c r="J52" s="61"/>
+      <c r="K52" s="61"/>
+      <c r="L52" s="61"/>
+      <c r="M52" s="61"/>
     </row>
     <row r="53" spans="1:13" ht="50.75">
       <c r="A53" s="18" t="s">
@@ -4613,13 +4073,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="G11:G16">
-    <cfRule type="containsText" dxfId="101" priority="149" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="47" priority="149" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="100" priority="150" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="46" priority="150" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",G11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="99" priority="151" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="45" priority="151" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G11)))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="152">
@@ -4634,13 +4094,13 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G18:G26">
-    <cfRule type="containsText" dxfId="98" priority="161" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="44" priority="161" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G18)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="97" priority="162" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="43" priority="162" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",G18)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="96" priority="163" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="42" priority="163" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G18)))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="164">
@@ -4655,6 +4115,15 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G34:G50">
+    <cfRule type="containsText" dxfId="41" priority="25" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",G34)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="40" priority="26" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",G34)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="39" priority="27" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",G34)))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="28">
       <colorScale>
         <cfvo type="min"/>
@@ -4664,17 +4133,6 @@
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G34:G50">
-    <cfRule type="containsText" dxfId="26" priority="25" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G34)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="25" priority="26" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G34)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="27" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G34)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53">
@@ -4689,14 +4147,14 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G53">
-    <cfRule type="containsText" dxfId="23" priority="21" operator="containsText" text="Pass">
+  <conditionalFormatting sqref="G53:G67">
+    <cfRule type="containsText" dxfId="38" priority="5" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G53)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="22" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="37" priority="6" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",G53)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="23" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="36" priority="7" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G53)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4712,15 +4170,16 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G54:G56">
-    <cfRule type="containsText" dxfId="20" priority="17" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G54)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="19" priority="18" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G54)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="19" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G54)))</formula>
+  <conditionalFormatting sqref="G57:G64">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G65">
@@ -4735,17 +4194,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G65">
-    <cfRule type="containsText" dxfId="17" priority="13" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G65)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="14" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G65)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="15" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G65)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="G66:G67">
     <cfRule type="colorScale" priority="12">
       <colorScale>
@@ -4758,41 +4206,16 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G66:G67">
-    <cfRule type="containsText" dxfId="14" priority="9" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G66)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="10" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G66)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="11" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G66)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G57:G64">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G57:G64">
-    <cfRule type="containsText" dxfId="11" priority="5" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G57)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G57)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G57)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J53:J67">
+    <cfRule type="containsText" dxfId="35" priority="1" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",J53)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",J53)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="33" priority="3" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",J53)))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -4802,17 +4225,6 @@
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J53:J67">
-    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",J53)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",J53)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",J53)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -4849,25 +4261,25 @@
       <c r="A1" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
     </row>
     <row r="2" spans="1:6" ht="16.899999999999999">
       <c r="A2" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
     </row>
     <row r="3" spans="1:6" ht="16.899999999999999">
       <c r="A3" s="39"/>
@@ -4895,7 +4307,7 @@
         <v>26</v>
       </c>
       <c r="C4" s="39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" s="39">
         <v>0</v>
@@ -4928,64 +4340,64 @@
       </c>
     </row>
     <row r="30" spans="1:13" ht="16.899999999999999">
-      <c r="A30" s="61" t="s">
+      <c r="A30" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="B30" s="61" t="s">
+      <c r="B30" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="C30" s="61" t="s">
+      <c r="C30" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="D30" s="61" t="s">
+      <c r="D30" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="E30" s="61" t="s">
+      <c r="E30" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="F30" s="61" t="s">
+      <c r="F30" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="G30" s="61" t="s">
+      <c r="G30" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="H30" s="61"/>
-      <c r="I30" s="61"/>
-      <c r="J30" s="61" t="s">
+      <c r="H30" s="62"/>
+      <c r="I30" s="62"/>
+      <c r="J30" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="K30" s="61"/>
-      <c r="L30" s="61"/>
-      <c r="M30" s="61" t="s">
+      <c r="K30" s="62"/>
+      <c r="L30" s="62"/>
+      <c r="M30" s="62" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="16.899999999999999">
-      <c r="A31" s="61"/>
-      <c r="B31" s="61"/>
-      <c r="C31" s="61"/>
-      <c r="D31" s="61"/>
-      <c r="E31" s="61"/>
-      <c r="F31" s="61"/>
-      <c r="G31" s="61" t="s">
+      <c r="A31" s="62"/>
+      <c r="B31" s="62"/>
+      <c r="C31" s="62"/>
+      <c r="D31" s="62"/>
+      <c r="E31" s="62"/>
+      <c r="F31" s="62"/>
+      <c r="G31" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="H31" s="61"/>
-      <c r="I31" s="61"/>
-      <c r="J31" s="61" t="s">
+      <c r="H31" s="62"/>
+      <c r="I31" s="62"/>
+      <c r="J31" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="K31" s="61"/>
-      <c r="L31" s="61"/>
-      <c r="M31" s="61"/>
+      <c r="K31" s="62"/>
+      <c r="L31" s="62"/>
+      <c r="M31" s="62"/>
     </row>
     <row r="32" spans="1:13" ht="50.75">
-      <c r="A32" s="61"/>
-      <c r="B32" s="61"/>
-      <c r="C32" s="61"/>
-      <c r="D32" s="61"/>
-      <c r="E32" s="61"/>
-      <c r="F32" s="61"/>
+      <c r="A32" s="62"/>
+      <c r="B32" s="62"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="62"/>
       <c r="G32" s="24" t="s">
         <v>20</v>
       </c>
@@ -5004,24 +4416,24 @@
       <c r="L32" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="M32" s="61"/>
+      <c r="M32" s="62"/>
     </row>
     <row r="33" spans="1:13" ht="16.899999999999999">
-      <c r="A33" s="59" t="s">
+      <c r="A33" s="60" t="s">
         <v>148</v>
       </c>
-      <c r="B33" s="59"/>
-      <c r="C33" s="59"/>
-      <c r="D33" s="59"/>
-      <c r="E33" s="59"/>
-      <c r="F33" s="59"/>
-      <c r="G33" s="59"/>
-      <c r="H33" s="59"/>
-      <c r="I33" s="59"/>
-      <c r="J33" s="59"/>
-      <c r="K33" s="59"/>
-      <c r="L33" s="59"/>
-      <c r="M33" s="59"/>
+      <c r="B33" s="60"/>
+      <c r="C33" s="60"/>
+      <c r="D33" s="60"/>
+      <c r="E33" s="60"/>
+      <c r="F33" s="60"/>
+      <c r="G33" s="60"/>
+      <c r="H33" s="60"/>
+      <c r="I33" s="60"/>
+      <c r="J33" s="60"/>
+      <c r="K33" s="60"/>
+      <c r="L33" s="60"/>
+      <c r="M33" s="60"/>
     </row>
     <row r="34" spans="1:13" ht="67.650000000000006">
       <c r="A34" s="22" t="s">
@@ -5041,7 +4453,7 @@
       <c r="G34" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H34" s="78" t="s">
+      <c r="H34" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I34" s="35" t="s">
@@ -5070,7 +4482,7 @@
       <c r="G35" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H35" s="78" t="s">
+      <c r="H35" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I35" s="35" t="s">
@@ -5099,7 +4511,7 @@
       <c r="G36" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H36" s="78" t="s">
+      <c r="H36" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I36" s="35" t="s">
@@ -5128,7 +4540,7 @@
       <c r="G37" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H37" s="78" t="s">
+      <c r="H37" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I37" s="35" t="s">
@@ -5157,7 +4569,7 @@
       <c r="G38" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H38" s="78" t="s">
+      <c r="H38" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I38" s="35" t="s">
@@ -5186,7 +4598,7 @@
       <c r="G39" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H39" s="78" t="s">
+      <c r="H39" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I39" s="35" t="s">
@@ -5215,7 +4627,7 @@
       <c r="G40" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H40" s="78" t="s">
+      <c r="H40" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I40" s="35" t="s">
@@ -5244,7 +4656,7 @@
       <c r="G41" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H41" s="78" t="s">
+      <c r="H41" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I41" s="35" t="s">
@@ -5273,7 +4685,7 @@
       <c r="G42" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H42" s="78" t="s">
+      <c r="H42" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I42" s="35" t="s">
@@ -5302,7 +4714,7 @@
       <c r="G43" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H43" s="78" t="s">
+      <c r="H43" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I43" s="35" t="s">
@@ -5331,7 +4743,7 @@
       <c r="G44" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H44" s="78" t="s">
+      <c r="H44" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I44" s="35" t="s">
@@ -5360,7 +4772,7 @@
       <c r="G45" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="H45" s="78" t="s">
+      <c r="H45" s="49" t="s">
         <v>54</v>
       </c>
       <c r="I45" s="35" t="s">
@@ -5372,21 +4784,21 @@
       <c r="M45" s="12"/>
     </row>
     <row r="47" spans="1:13" ht="16.899999999999999">
-      <c r="A47" s="60" t="s">
+      <c r="A47" s="61" t="s">
         <v>172</v>
       </c>
-      <c r="B47" s="60"/>
-      <c r="C47" s="60"/>
-      <c r="D47" s="60"/>
-      <c r="E47" s="60"/>
-      <c r="F47" s="60"/>
-      <c r="G47" s="60"/>
-      <c r="H47" s="60"/>
-      <c r="I47" s="60"/>
-      <c r="J47" s="60"/>
-      <c r="K47" s="60"/>
-      <c r="L47" s="60"/>
-      <c r="M47" s="60"/>
+      <c r="B47" s="61"/>
+      <c r="C47" s="61"/>
+      <c r="D47" s="61"/>
+      <c r="E47" s="61"/>
+      <c r="F47" s="61"/>
+      <c r="G47" s="61"/>
+      <c r="H47" s="61"/>
+      <c r="I47" s="61"/>
+      <c r="J47" s="61"/>
+      <c r="K47" s="61"/>
+      <c r="L47" s="61"/>
+      <c r="M47" s="61"/>
     </row>
     <row r="48" spans="1:13" ht="114.6" customHeight="1">
       <c r="A48" s="18" t="s">
@@ -5889,13 +5301,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="G11:G22">
-    <cfRule type="containsText" dxfId="83" priority="145" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="32" priority="145" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="82" priority="146" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="31" priority="146" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",G11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="81" priority="147" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="30" priority="147" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G11)))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="148">
@@ -5910,13 +5322,13 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G24:G32">
-    <cfRule type="containsText" dxfId="80" priority="149" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="29" priority="149" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G24)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="79" priority="150" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="28" priority="150" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",G24)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="78" priority="151" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="27" priority="151" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G24)))</formula>
     </cfRule>
     <cfRule type="colorScale" priority="152">
@@ -5931,6 +5343,15 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G34:G45">
+    <cfRule type="containsText" dxfId="26" priority="17" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",G34)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="25" priority="18" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",G34)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="24" priority="19" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",G34)))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
@@ -5940,17 +5361,6 @@
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G34:G45">
-    <cfRule type="containsText" dxfId="41" priority="17" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G34)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="40" priority="18" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G34)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="39" priority="19" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G34)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G48:G57">
@@ -5965,15 +5375,27 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G48:G57">
-    <cfRule type="containsText" dxfId="38" priority="13" operator="containsText" text="Pass">
+  <conditionalFormatting sqref="G48:G60">
+    <cfRule type="containsText" dxfId="23" priority="5" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G48)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="37" priority="14" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="22" priority="6" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",G48)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="36" priority="15" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="21" priority="7" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G48)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G58">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G59:G60">
@@ -5988,41 +5410,16 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G59:G60">
-    <cfRule type="containsText" dxfId="35" priority="9" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G59)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="34" priority="10" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G59)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="33" priority="11" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G59)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G58">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G58">
-    <cfRule type="containsText" dxfId="32" priority="5" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G58)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="31" priority="6" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G58)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="7" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G58)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J48:J60">
+    <cfRule type="containsText" dxfId="20" priority="1" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",J48)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="19" priority="2" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",J48)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="18" priority="3" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",J48)))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -6032,17 +5429,6 @@
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J48:J60">
-    <cfRule type="containsText" dxfId="29" priority="1" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",J48)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="28" priority="2" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",J48)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="27" priority="3" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",J48)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -6084,13 +5470,13 @@
       <c r="A1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
       <c r="G1" s="10"/>
       <c r="H1" s="25"/>
       <c r="J1" s="10"/>
@@ -6099,13 +5485,13 @@
       <c r="A2" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="78" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
       <c r="G2" s="10"/>
       <c r="H2" s="25"/>
       <c r="J2" s="10"/>
@@ -6190,64 +5576,64 @@
       <c r="J6" s="10"/>
     </row>
     <row r="7" spans="1:13" s="19" customFormat="1">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="74" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="73" t="s">
+      <c r="B7" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="73" t="s">
+      <c r="C7" s="74" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="73" t="s">
+      <c r="D7" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="73" t="s">
+      <c r="E7" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="73" t="s">
+      <c r="F7" s="74" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="70" t="s">
+      <c r="G7" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="71"/>
-      <c r="I7" s="72"/>
-      <c r="J7" s="70" t="s">
+      <c r="H7" s="72"/>
+      <c r="I7" s="73"/>
+      <c r="J7" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="K7" s="71"/>
-      <c r="L7" s="72"/>
-      <c r="M7" s="73" t="s">
+      <c r="K7" s="72"/>
+      <c r="L7" s="73"/>
+      <c r="M7" s="74" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:13" s="19" customFormat="1">
-      <c r="A8" s="74"/>
-      <c r="B8" s="74"/>
-      <c r="C8" s="74"/>
-      <c r="D8" s="74"/>
-      <c r="E8" s="74"/>
-      <c r="F8" s="74"/>
-      <c r="G8" s="70" t="s">
+      <c r="A8" s="75"/>
+      <c r="B8" s="75"/>
+      <c r="C8" s="75"/>
+      <c r="D8" s="75"/>
+      <c r="E8" s="75"/>
+      <c r="F8" s="75"/>
+      <c r="G8" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="71"/>
-      <c r="I8" s="72"/>
-      <c r="J8" s="70" t="s">
+      <c r="H8" s="72"/>
+      <c r="I8" s="73"/>
+      <c r="J8" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="K8" s="71"/>
-      <c r="L8" s="72"/>
-      <c r="M8" s="74"/>
+      <c r="K8" s="72"/>
+      <c r="L8" s="73"/>
+      <c r="M8" s="75"/>
     </row>
     <row r="9" spans="1:13" s="19" customFormat="1">
-      <c r="A9" s="75"/>
-      <c r="B9" s="75"/>
-      <c r="C9" s="75"/>
-      <c r="D9" s="75"/>
-      <c r="E9" s="75"/>
-      <c r="F9" s="75"/>
+      <c r="A9" s="76"/>
+      <c r="B9" s="76"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
+      <c r="F9" s="76"/>
       <c r="G9" s="24" t="s">
         <v>20</v>
       </c>
@@ -6266,24 +5652,24 @@
       <c r="L9" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="M9" s="75"/>
+      <c r="M9" s="76"/>
     </row>
     <row r="10" spans="1:13" s="19" customFormat="1">
-      <c r="A10" s="64" t="s">
+      <c r="A10" s="65" t="s">
         <v>216</v>
       </c>
-      <c r="B10" s="65"/>
-      <c r="C10" s="65"/>
-      <c r="D10" s="65"/>
-      <c r="E10" s="65"/>
-      <c r="F10" s="65"/>
-      <c r="G10" s="65"/>
-      <c r="H10" s="65"/>
-      <c r="I10" s="65"/>
-      <c r="J10" s="65"/>
-      <c r="K10" s="65"/>
-      <c r="L10" s="65"/>
-      <c r="M10" s="66"/>
+      <c r="B10" s="66"/>
+      <c r="C10" s="66"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="66"/>
+      <c r="G10" s="66"/>
+      <c r="H10" s="66"/>
+      <c r="I10" s="66"/>
+      <c r="J10" s="66"/>
+      <c r="K10" s="66"/>
+      <c r="L10" s="66"/>
+      <c r="M10" s="67"/>
     </row>
     <row r="11" spans="1:13" s="19" customFormat="1" ht="33.85">
       <c r="A11" s="22" t="s">
@@ -6518,21 +5904,21 @@
       <c r="M18" s="12"/>
     </row>
     <row r="19" spans="1:13" s="19" customFormat="1">
-      <c r="A19" s="67" t="s">
+      <c r="A19" s="68" t="s">
         <v>225</v>
       </c>
-      <c r="B19" s="68"/>
-      <c r="C19" s="68"/>
-      <c r="D19" s="68"/>
-      <c r="E19" s="68"/>
-      <c r="F19" s="68"/>
-      <c r="G19" s="68"/>
-      <c r="H19" s="68"/>
-      <c r="I19" s="68"/>
-      <c r="J19" s="68"/>
-      <c r="K19" s="68"/>
-      <c r="L19" s="68"/>
-      <c r="M19" s="69"/>
+      <c r="B19" s="69"/>
+      <c r="C19" s="69"/>
+      <c r="D19" s="69"/>
+      <c r="E19" s="69"/>
+      <c r="F19" s="69"/>
+      <c r="G19" s="69"/>
+      <c r="H19" s="69"/>
+      <c r="I19" s="69"/>
+      <c r="J19" s="69"/>
+      <c r="K19" s="69"/>
+      <c r="L19" s="69"/>
+      <c r="M19" s="70"/>
     </row>
     <row r="20" spans="1:13" s="19" customFormat="1" ht="50.75">
       <c r="A20" s="18" t="s">
@@ -6917,13 +6303,13 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G18">
-    <cfRule type="containsText" dxfId="68" priority="10" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="17" priority="10" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="67" priority="11" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="16" priority="11" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",G11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="66" priority="12" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="15" priority="12" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G11)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6976,13 +6362,13 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G20:G28">
-    <cfRule type="containsText" dxfId="65" priority="6" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="14" priority="6" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G20)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="64" priority="7" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="13" priority="7" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",G20)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="63" priority="8" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="12" priority="8" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G20)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7011,13 +6397,13 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J20:J28">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",J20)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="10" priority="2" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",J20)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",J20)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7072,13 +6458,13 @@
       <c r="A1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
       <c r="G1" s="10"/>
       <c r="H1" s="25"/>
       <c r="J1" s="10"/>
@@ -7087,13 +6473,13 @@
       <c r="A2" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="78" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
       <c r="G2" s="10"/>
       <c r="H2" s="25"/>
       <c r="J2" s="10"/>
@@ -7149,10 +6535,10 @@
         <v>11</v>
       </c>
       <c r="B5" s="28">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C5" s="28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="30">
         <f>COUNTIF(J11:J20,"Untested")</f>
@@ -7163,7 +6549,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="28">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G5" s="10"/>
       <c r="H5" s="25"/>
@@ -7178,64 +6564,64 @@
       <c r="J6" s="10"/>
     </row>
     <row r="7" spans="1:13" s="19" customFormat="1">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="61" t="s">
+      <c r="B7" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="61" t="s">
+      <c r="F7" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="61" t="s">
+      <c r="G7" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="61"/>
-      <c r="I7" s="61"/>
-      <c r="J7" s="61" t="s">
+      <c r="H7" s="62"/>
+      <c r="I7" s="62"/>
+      <c r="J7" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="K7" s="61"/>
-      <c r="L7" s="61"/>
-      <c r="M7" s="61" t="s">
+      <c r="K7" s="62"/>
+      <c r="L7" s="62"/>
+      <c r="M7" s="62" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:13" s="19" customFormat="1">
-      <c r="A8" s="61"/>
-      <c r="B8" s="61"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61" t="s">
+      <c r="A8" s="62"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="61"/>
-      <c r="I8" s="61"/>
-      <c r="J8" s="61" t="s">
+      <c r="H8" s="62"/>
+      <c r="I8" s="62"/>
+      <c r="J8" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="K8" s="61"/>
-      <c r="L8" s="61"/>
-      <c r="M8" s="61"/>
+      <c r="K8" s="62"/>
+      <c r="L8" s="62"/>
+      <c r="M8" s="62"/>
     </row>
     <row r="9" spans="1:13" s="19" customFormat="1">
-      <c r="A9" s="61"/>
-      <c r="B9" s="61"/>
-      <c r="C9" s="61"/>
-      <c r="D9" s="61"/>
-      <c r="E9" s="61"/>
-      <c r="F9" s="61"/>
+      <c r="A9" s="62"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="62"/>
       <c r="G9" s="24" t="s">
         <v>20</v>
       </c>
@@ -7254,24 +6640,24 @@
       <c r="L9" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="M9" s="61"/>
+      <c r="M9" s="62"/>
     </row>
     <row r="10" spans="1:13" s="19" customFormat="1">
-      <c r="A10" s="59" t="s">
+      <c r="A10" s="60" t="s">
         <v>271</v>
       </c>
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="59"/>
-      <c r="I10" s="59"/>
-      <c r="J10" s="59"/>
-      <c r="K10" s="59"/>
-      <c r="L10" s="59"/>
-      <c r="M10" s="59"/>
+      <c r="B10" s="60"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
+      <c r="H10" s="60"/>
+      <c r="I10" s="60"/>
+      <c r="J10" s="60"/>
+      <c r="K10" s="60"/>
+      <c r="L10" s="60"/>
+      <c r="M10" s="60"/>
     </row>
     <row r="11" spans="1:13" s="19" customFormat="1" ht="33.85">
       <c r="A11" s="22" t="s">
@@ -7403,21 +6789,21 @@
       <c r="M15" s="12"/>
     </row>
     <row r="16" spans="1:13" s="19" customFormat="1">
-      <c r="A16" s="60" t="s">
+      <c r="A16" s="61" t="s">
         <v>277</v>
       </c>
-      <c r="B16" s="60"/>
-      <c r="C16" s="60"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
-      <c r="G16" s="60"/>
-      <c r="H16" s="60"/>
-      <c r="I16" s="60"/>
-      <c r="J16" s="60"/>
-      <c r="K16" s="60"/>
-      <c r="L16" s="60"/>
-      <c r="M16" s="60"/>
+      <c r="B16" s="61"/>
+      <c r="C16" s="61"/>
+      <c r="D16" s="61"/>
+      <c r="E16" s="61"/>
+      <c r="F16" s="61"/>
+      <c r="G16" s="61"/>
+      <c r="H16" s="61"/>
+      <c r="I16" s="61"/>
+      <c r="J16" s="61"/>
+      <c r="K16" s="61"/>
+      <c r="L16" s="61"/>
+      <c r="M16" s="61"/>
     </row>
     <row r="17" spans="1:13" s="19" customFormat="1" ht="67.650000000000006">
       <c r="A17" s="18" t="s">
@@ -7712,6 +7098,15 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="G11:G15">
+    <cfRule type="containsText" dxfId="8" priority="17" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",G11)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="7" priority="18" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",G11)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="6" priority="19" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",G11)))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
@@ -7721,17 +7116,6 @@
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G15">
-    <cfRule type="containsText" dxfId="53" priority="17" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G11)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="52" priority="18" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G11)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="51" priority="19" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G11)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G17:G21">
@@ -7746,15 +7130,27 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G17:G21">
-    <cfRule type="containsText" dxfId="50" priority="13" operator="containsText" text="Pass">
+  <conditionalFormatting sqref="G17:G23">
+    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G17)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="49" priority="14" operator="containsText" text="Fail">
+    <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="Fail">
       <formula>NOT(ISERROR(SEARCH("Fail",G17)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="48" priority="15" operator="containsText" text="Pass">
+    <cfRule type="containsText" dxfId="3" priority="7" operator="containsText" text="Pass">
       <formula>NOT(ISERROR(SEARCH("Pass",G17)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G22">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G23">
@@ -7769,41 +7165,16 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G23">
-    <cfRule type="containsText" dxfId="47" priority="9" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G23)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="46" priority="10" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G23)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="45" priority="11" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G23)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G22">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G22">
-    <cfRule type="containsText" dxfId="44" priority="5" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G22)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="43" priority="6" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",G22)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="42" priority="7" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",G22)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J17:J23">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",J17)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Fail">
+      <formula>NOT(ISERROR(SEARCH("Fail",J17)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Pass">
+      <formula>NOT(ISERROR(SEARCH("Pass",J17)))</formula>
+    </cfRule>
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -7813,17 +7184,6 @@
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J17:J23">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",J17)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Fail">
-      <formula>NOT(ISERROR(SEARCH("Fail",J17)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Pass">
-      <formula>NOT(ISERROR(SEARCH("Pass",J17)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">

</xml_diff>